<commit_message>
nii-frontier engine-v2: curve as sole named object - RatesCurve reads scenario+holiday ranges directly, stores provenance, strip now includes dayFactor + accumFactor; GET spills header + full strip; drop separate HolidayTable/FedScenario classes; 3 .bas modules; golden values reverified
</commit_message>
<xml_diff>
--- a/projects/nii-frontier/engine-v2/NII_Engine_v2.xlsx
+++ b/projects/nii-frontier/engine-v2/NII_Engine_v2.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NII ENGINE v2 — object layer</t>
+          <t>NII ENGINE v2 — curve as the named object</t>
         </is>
       </c>
     </row>
@@ -505,125 +505,128 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Six functions:</t>
+          <t>Four functions:</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  HolidayTable(name, range)         build a named holiday set</t>
+          <t xml:space="preserve">  RatesCurve(name,start,end,sofr,scenRange,holRange)  build the curve</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FedScenario(name, range)          build a named FOMC move list</t>
+          <t xml:space="preserve">  GET(curveCell)            spill the curve: provenance + daily strip</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  RatesCurve(name,start,end,sofr,scenCell,holCell)   assemble the curve</t>
+          <t xml:space="preserve">  ACCRUE(start,end,amount,type,curveCell)             interest $mm</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GET(handleCell)                   spill an object's whole dataset</t>
+          <t xml:space="preserve">  SWAP(start,end,notional,fixed,curveCell,leg)        FIXED|FLOAT|NET</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ACCRUE(start,end,amount,type,curveCell)            interest $mm</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SWAP(start,end,notional,fixed,curveCell,leg)       FIXED|FLOAT|NET</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>The curve is the one named object. It reads the scenario and holiday</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ranges directly, records which ranges built it (provenance), and stores</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>the daily strip: date | rate% | dayFactor | accumFactor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>SETUP</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>1. Alt+F11. Import the 6 files from the bas folder:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   File &gt; Import File...  (mRegistry, cHolidayTable, cFedScenario,</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   cRatesCurve, mEngine — classes import as class modules automatically).</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1. Alt+F11 &gt; File &gt; Import File... import the 3 .bas from bas/</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>2. Save as .xlsm. Press Ctrl+Alt+F9.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (mRegistry, cRatesCurve, mEngine).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>2. Save as .xlsm. Press Ctrl+Alt+F9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>3. MODEL sheet: paste each column-E formula into the yellow cell.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Order matters: B4 holidays, B5 scenario, B6 curve, THEN the rest.</t>
-        </is>
-      </c>
-    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>4. Results should match the Expected column; GET cells spill a table.</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Build the curve (B6) first; the rest reference it.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>4. Results should match Expected; GET($B$6) spills the strip.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>RULE: every handle is passed as a CELL ($B$6), never as typed text,</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>so editing an input cascades through the whole chain automatically.</t>
+          <t>RULE: scenRange, holRange and curveCell are passed as RANGES/CELLS,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>never as typed text, so editing inputs cascades automatically.</t>
         </is>
       </c>
     </row>
@@ -768,7 +771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -788,37 +791,13 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>1 · BUILD OBJECTS (in this order)</t>
+          <t>1 · BUILD THE CURVE (reads the input ranges directly)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>PASTE THIS</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Holidays</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="E4" s="3">
-        <f>HolidayTable("HOL_US",INPUTS!A4:B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="E5" s="3">
-        <f>FedScenario("CUT",INPUTS!D4:E7)</f>
-        <v/>
       </c>
     </row>
     <row r="6">
@@ -829,7 +808,7 @@
       </c>
       <c r="B6" s="10" t="n"/>
       <c r="E6" s="3">
-        <f>RatesCurve("curve1",DATE(2026,6,15),DATE(2030,12,31),3.80,$B$5,$B$4)</f>
+        <f>RatesCurve("curve1",DATE(2026,6,15),DATE(2030,12,31),3.80,INPUTS!D4:E7,INPUTS!A4:B9)</f>
         <v/>
       </c>
     </row>
@@ -960,47 +939,32 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>4 · INSPECT (GET spills the whole dataset)</t>
+          <t>4 · INSPECT — GET spills provenance + the daily strip</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Holidays</t>
+          <t>Curve table</t>
         </is>
       </c>
       <c r="E18" s="3">
-        <f>GET($B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="E19" s="3">
-        <f>GET($B$5)</f>
+        <f>GET($B$6)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Curve strip</t>
-        </is>
-      </c>
-      <c r="E20" s="3">
-        <f>GET($B$6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>GET spills into the cells below/right of it — give it empty room.</t>
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Spills: header (curve/SOFR), then date | rate% | dayFactor | accumFactor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Give it empty room below and to the right.</t>
         </is>
       </c>
     </row>

</xml_diff>